<commit_message>
feat(dp): planilha ganha horario de entrada/saida observado + colunas p/ o horario correto
Jordan: 'coloque a coluna de horario que os funcionarios entram e saem, pois varia tambem
de condominio para condominio'. Confirmado no dado — Ideal Flores sozinho vai de
04:00->17:00 a 16:00->05:00.

Horario HABITUAL e nao media: media de horario nao significa nada quando o turno atravessa
a meia-noite (07:00 e 19:00 dariam 13:00, que ninguem trabalha). Uso a MODA da hora, com a
faixa observada ao lado para mostrar dispersao.

19 colunas, 5 para o Jordan preencher (intrajornada, batidas, entrada, saida, observacao).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/auditoria/ponto_intrajornada_conferencia.xlsx
+++ b/auditoria/ponto_intrajornada_conferencia.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N56"/>
+  <dimension ref="A1:S57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -458,10 +458,15 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="34" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
     <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="34" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -521,22 +526,52 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Entrada
+habitual</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Saída
+habitual</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Faixa de entrada
+observada</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Divergência</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>→ RECEBE INTRAJORNADA?
 (preencher: SIM / NAO)</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>→ Quantas batidas por turno?
 (preencher: 2 / 4)</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>→ Horário CORRETO
+entrada (ex.: 07:00)</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>→ Horário CORRETO
+saída (ex.: 19:00)</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>→ Observação</t>
         </is>
@@ -591,12 +626,29 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>05:00–21:47</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
           <t>cadastro diz NÃO mas bate 1.1×/dia · folha não pagou mas bate 1.1×/dia</t>
         </is>
       </c>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3" t="n"/>
+      <c r="O2" s="3" t="n"/>
+      <c r="P2" s="3" t="n"/>
+      <c r="Q2" s="3" t="n"/>
+      <c r="R2" s="3" t="n"/>
+      <c r="S2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -645,7 +697,22 @@
       <c r="J3" t="n">
         <v>3</v>
       </c>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -696,12 +763,29 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>00:00–22:24</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
           <t>cadastro diz NÃO mas bate 2.0×/dia · folha não pagou mas bate 2.0×/dia</t>
         </is>
       </c>
-      <c r="L4" s="3" t="n"/>
-      <c r="M4" s="3" t="n"/>
-      <c r="N4" s="3" t="n"/>
+      <c r="O4" s="3" t="n"/>
+      <c r="P4" s="3" t="n"/>
+      <c r="Q4" s="3" t="n"/>
+      <c r="R4" s="3" t="n"/>
+      <c r="S4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -752,12 +836,29 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>00:42–20:51</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
           <t>cadastro diz NÃO mas bate 2.0×/dia · folha não pagou mas bate 2.0×/dia</t>
         </is>
       </c>
-      <c r="L5" s="3" t="n"/>
-      <c r="M5" s="3" t="n"/>
-      <c r="N5" s="3" t="n"/>
+      <c r="O5" s="3" t="n"/>
+      <c r="P5" s="3" t="n"/>
+      <c r="Q5" s="3" t="n"/>
+      <c r="R5" s="3" t="n"/>
+      <c r="S5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -806,7 +907,22 @@
       <c r="J6" t="n">
         <v>4</v>
       </c>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>05:00–09:27</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -855,7 +971,22 @@
       <c r="J7" t="n">
         <v>17</v>
       </c>
-      <c r="K7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>04:41–12:20</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -906,12 +1037,29 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>00:00–20:50</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
           <t>folha não pagou mas bate 2.2×/dia · cadastro e folha discordam</t>
         </is>
       </c>
-      <c r="L8" s="3" t="n"/>
-      <c r="M8" s="3" t="n"/>
-      <c r="N8" s="3" t="n"/>
+      <c r="O8" s="3" t="n"/>
+      <c r="P8" s="3" t="n"/>
+      <c r="Q8" s="3" t="n"/>
+      <c r="R8" s="3" t="n"/>
+      <c r="S8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -960,7 +1108,22 @@
       <c r="J9" t="n">
         <v>30</v>
       </c>
-      <c r="K9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>07:00–11:00</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1009,7 +1172,22 @@
       <c r="J10" t="n">
         <v>28</v>
       </c>
-      <c r="K10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>07:00–11:08</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1058,7 +1236,22 @@
       <c r="J11" t="n">
         <v>30</v>
       </c>
-      <c r="K11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>07:00–11:00</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1107,7 +1300,22 @@
       <c r="J12" t="n">
         <v>9</v>
       </c>
-      <c r="K12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>07:00–14:47</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1156,7 +1364,22 @@
       <c r="J13" t="n">
         <v>24</v>
       </c>
-      <c r="K13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>07:00–11:00</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1205,7 +1428,22 @@
       <c r="J14" t="n">
         <v>6</v>
       </c>
-      <c r="K14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>04:58–16:03</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1256,12 +1494,29 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
+          <t>01:00</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>01:00–22:00</t>
+        </is>
+      </c>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
           <t>cadastro diz NÃO mas bate 1.9×/dia · folha não pagou mas bate 1.9×/dia</t>
         </is>
       </c>
-      <c r="L15" s="3" t="n"/>
-      <c r="M15" s="3" t="n"/>
-      <c r="N15" s="3" t="n"/>
+      <c r="O15" s="3" t="n"/>
+      <c r="P15" s="3" t="n"/>
+      <c r="Q15" s="3" t="n"/>
+      <c r="R15" s="3" t="n"/>
+      <c r="S15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1312,12 +1567,29 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>00:00–22:01</t>
+        </is>
+      </c>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
           <t>cadastro diz NÃO mas bate 1.9×/dia · folha não pagou mas bate 1.9×/dia</t>
         </is>
       </c>
-      <c r="L16" s="3" t="n"/>
-      <c r="M16" s="3" t="n"/>
-      <c r="N16" s="3" t="n"/>
+      <c r="O16" s="3" t="n"/>
+      <c r="P16" s="3" t="n"/>
+      <c r="Q16" s="3" t="n"/>
+      <c r="R16" s="3" t="n"/>
+      <c r="S16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1368,12 +1640,29 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>02:00–22:00</t>
+        </is>
+      </c>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
           <t>cadastro diz NÃO mas bate 2.0×/dia · folha não pagou mas bate 2.0×/dia</t>
         </is>
       </c>
-      <c r="L17" s="3" t="n"/>
-      <c r="M17" s="3" t="n"/>
-      <c r="N17" s="3" t="n"/>
+      <c r="O17" s="3" t="n"/>
+      <c r="P17" s="3" t="n"/>
+      <c r="Q17" s="3" t="n"/>
+      <c r="R17" s="3" t="n"/>
+      <c r="S17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1424,12 +1713,29 @@
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>05:56–10:09</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
           <t>cadastro diz SIM mas bate 3.4×/dia · cadastro e folha discordam</t>
         </is>
       </c>
-      <c r="L18" s="3" t="n"/>
-      <c r="M18" s="3" t="n"/>
-      <c r="N18" s="3" t="n"/>
+      <c r="O18" s="3" t="n"/>
+      <c r="P18" s="3" t="n"/>
+      <c r="Q18" s="3" t="n"/>
+      <c r="R18" s="3" t="n"/>
+      <c r="S18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1478,7 +1784,22 @@
       <c r="J19" t="n">
         <v>3</v>
       </c>
-      <c r="K19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1529,12 +1850,29 @@
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>05:00–10:00</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
           <t>cadastro diz SIM mas bate 4.0×/dia · cadastro e folha discordam</t>
         </is>
       </c>
-      <c r="L20" s="3" t="n"/>
-      <c r="M20" s="3" t="n"/>
-      <c r="N20" s="3" t="n"/>
+      <c r="O20" s="3" t="n"/>
+      <c r="P20" s="3" t="n"/>
+      <c r="Q20" s="3" t="n"/>
+      <c r="R20" s="3" t="n"/>
+      <c r="S20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1583,7 +1921,22 @@
       <c r="J21" t="n">
         <v>18</v>
       </c>
-      <c r="K21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>06:02–18:00</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1634,12 +1987,29 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>05:58–12:01</t>
+        </is>
+      </c>
+      <c r="N22" s="3" t="inlineStr">
+        <is>
           <t>cadastro diz SIM mas bate 3.9×/dia · cadastro e folha discordam</t>
         </is>
       </c>
-      <c r="L22" s="3" t="n"/>
-      <c r="M22" s="3" t="n"/>
-      <c r="N22" s="3" t="n"/>
+      <c r="O22" s="3" t="n"/>
+      <c r="P22" s="3" t="n"/>
+      <c r="Q22" s="3" t="n"/>
+      <c r="R22" s="3" t="n"/>
+      <c r="S22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1688,7 +2058,22 @@
       <c r="J23" t="n">
         <v>31</v>
       </c>
-      <c r="K23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>05:57–11:00</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1737,7 +2122,22 @@
       <c r="J24" t="n">
         <v>31</v>
       </c>
-      <c r="K24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>07:00–12:00</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1786,7 +2186,22 @@
       <c r="J25" t="n">
         <v>4</v>
       </c>
-      <c r="K25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>06:00–18:00</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -1837,12 +2252,29 @@
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>06:00–06:01</t>
+        </is>
+      </c>
+      <c r="N26" s="3" t="inlineStr">
+        <is>
           <t>cadastro diz NÃO mas bate 2.6×/dia · cadastro e folha discordam</t>
         </is>
       </c>
-      <c r="L26" s="3" t="n"/>
-      <c r="M26" s="3" t="n"/>
-      <c r="N26" s="3" t="n"/>
+      <c r="O26" s="3" t="n"/>
+      <c r="P26" s="3" t="n"/>
+      <c r="Q26" s="3" t="n"/>
+      <c r="R26" s="3" t="n"/>
+      <c r="S26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1891,7 +2323,22 @@
       <c r="J27" t="n">
         <v>4</v>
       </c>
-      <c r="K27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1940,7 +2387,22 @@
       <c r="J28" t="n">
         <v>34</v>
       </c>
-      <c r="K28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>05:52–22:00</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1989,7 +2451,22 @@
       <c r="J29" t="n">
         <v>19</v>
       </c>
-      <c r="K29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>00:51–12:51</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -2040,12 +2517,29 @@
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="L30" s="3" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>07:00–19:28</t>
+        </is>
+      </c>
+      <c r="N30" s="3" t="inlineStr">
+        <is>
           <t>folha pagou mas bate 3.9×/dia · cadastro e folha discordam</t>
         </is>
       </c>
-      <c r="L30" s="3" t="n"/>
-      <c r="M30" s="3" t="n"/>
-      <c r="N30" s="3" t="n"/>
+      <c r="O30" s="3" t="n"/>
+      <c r="P30" s="3" t="n"/>
+      <c r="Q30" s="3" t="n"/>
+      <c r="R30" s="3" t="n"/>
+      <c r="S30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2094,7 +2588,22 @@
       <c r="J31" t="n">
         <v>29</v>
       </c>
-      <c r="K31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>06:00–12:07</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -2145,12 +2654,29 @@
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="L32" s="3" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>06:00–12:00</t>
+        </is>
+      </c>
+      <c r="N32" s="3" t="inlineStr">
+        <is>
           <t>cadastro diz SIM mas bate 3.7×/dia · cadastro e folha discordam</t>
         </is>
       </c>
-      <c r="L32" s="3" t="n"/>
-      <c r="M32" s="3" t="n"/>
-      <c r="N32" s="3" t="n"/>
+      <c r="O32" s="3" t="n"/>
+      <c r="P32" s="3" t="n"/>
+      <c r="Q32" s="3" t="n"/>
+      <c r="R32" s="3" t="n"/>
+      <c r="S32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2199,7 +2725,22 @@
       <c r="J33" t="n">
         <v>9</v>
       </c>
-      <c r="K33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>00:57–10:02</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2248,7 +2789,22 @@
       <c r="J34" t="n">
         <v>8</v>
       </c>
-      <c r="K34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>05:00–17:00</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2297,7 +2853,22 @@
       <c r="J35" t="n">
         <v>13</v>
       </c>
-      <c r="K35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>04:57–16:50</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2346,7 +2917,22 @@
       <c r="J36" t="n">
         <v>15</v>
       </c>
-      <c r="K36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>05:00–09:00</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2395,7 +2981,22 @@
       <c r="J37" t="n">
         <v>24</v>
       </c>
-      <c r="K37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>00:00–21:03</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -2446,12 +3047,29 @@
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="L38" s="3" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>06:51–12:02</t>
+        </is>
+      </c>
+      <c r="N38" s="3" t="inlineStr">
+        <is>
           <t>cadastro diz NÃO mas bate 2.9×/dia · folha não pagou mas bate 2.9×/dia</t>
         </is>
       </c>
-      <c r="L38" s="3" t="n"/>
-      <c r="M38" s="3" t="n"/>
-      <c r="N38" s="3" t="n"/>
+      <c r="O38" s="3" t="n"/>
+      <c r="P38" s="3" t="n"/>
+      <c r="Q38" s="3" t="n"/>
+      <c r="R38" s="3" t="n"/>
+      <c r="S38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2500,7 +3118,22 @@
       <c r="J39" t="n">
         <v>30</v>
       </c>
-      <c r="K39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>07:00–16:02</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2549,7 +3182,22 @@
       <c r="J40" t="n">
         <v>27</v>
       </c>
-      <c r="K40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>04:58–21:01</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2598,7 +3246,22 @@
       <c r="J41" t="n">
         <v>17</v>
       </c>
-      <c r="K41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>05:00–09:00</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2647,7 +3310,22 @@
       <c r="J42" t="n">
         <v>33</v>
       </c>
-      <c r="K42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>00:54–21:01</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2696,7 +3374,22 @@
       <c r="J43" t="n">
         <v>18</v>
       </c>
-      <c r="K43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>05:00–09:00</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2745,7 +3438,22 @@
       <c r="J44" t="n">
         <v>29</v>
       </c>
-      <c r="K44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>06:59–16:07</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2794,7 +3502,22 @@
       <c r="J45" t="n">
         <v>32</v>
       </c>
-      <c r="K45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>07:00–11:00</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2843,7 +3566,22 @@
       <c r="J46" t="n">
         <v>33</v>
       </c>
-      <c r="K46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>04:49–20:50</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2892,7 +3630,22 @@
       <c r="J47" t="n">
         <v>34</v>
       </c>
-      <c r="K47" t="inlineStr"/>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>04:47–20:55</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2941,7 +3694,22 @@
       <c r="J48" t="n">
         <v>16</v>
       </c>
-      <c r="K48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>04:49–21:02</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2990,7 +3758,22 @@
       <c r="J49" t="n">
         <v>14</v>
       </c>
-      <c r="K49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>04:46–08:59</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3039,7 +3822,22 @@
       <c r="J50" t="n">
         <v>30</v>
       </c>
-      <c r="K50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>07:00–11:02</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3088,12 +3886,27 @@
       <c r="J51" t="n">
         <v>23</v>
       </c>
-      <c r="K51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>07:00–11:01</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>LEGENDA — as 3 últimas colunas (laranja) são para você preencher.</t>
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>LEGENDA — as 3 últimas colunas (laranja) são para você preencher (intrajornada, batidas, horário de entrada e saída, observação).</t>
         </is>
       </c>
     </row>
@@ -3113,6 +3926,13 @@
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Entrada/saída habitual = a hora que MAIS se repete nas batidas (moda), não a média — média não vale para turno que vira a meia-noite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
         <is>
           <t>Média cai abaixo do esperado quando falta batida — por isso o número vem com os dias, para você ver o peso da amostra.</t>
         </is>

</xml_diff>